<commit_message>
Add all scripts, figures, and core modules
</commit_message>
<xml_diff>
--- a/Supplementary_Materials_for_review/Supplementary_Tables.xlsx
+++ b/Supplementary_Materials_for_review/Supplementary_Tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tina/PycharmProjects/FcmR_IgM_Supplementary/Supplementary_Materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tina/PycharmProjects/FcmR_IgM_Supplementary/Supplementary_Materials_for_review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F338A6-C1FC-FB4B-BF48-C9149FBDC8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1521ACCE-1B25-5645-87CC-BC1CB0FEEB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16920" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table S1" sheetId="1" r:id="rId1"/>
@@ -330,7 +330,7 @@
     <numFmt numFmtId="177" formatCode="0.000_ "/>
     <numFmt numFmtId="178" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,12 +378,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="宋体"/>
@@ -394,15 +388,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <vertAlign val="subscript"/>
@@ -427,7 +412,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -455,11 +440,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -491,24 +485,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -530,30 +515,52 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -857,7 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="13" width="16.83203125" style="4" customWidth="1"/>
@@ -865,21 +872,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="2" customFormat="1" ht="12" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" ht="12" customHeight="1">
       <c r="A2" s="7"/>
@@ -897,43 +904,43 @@
       <c r="M2" s="7"/>
     </row>
     <row r="3" spans="1:13" s="3" customFormat="1" ht="12" customHeight="1">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="24" t="s">
+      <c r="J3" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="K3" s="24" t="s">
+      <c r="K3" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="L3" s="24" t="s">
+      <c r="L3" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="M3" s="24" t="s">
+      <c r="M3" s="21" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1061,68 +1068,108 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="3" customFormat="1" ht="12" customHeight="1">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="31">
         <v>1.21</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="31">
         <v>1.1739999999999999</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="31">
         <v>1.2470000000000001</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="31">
         <v>2.4929999999999999</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="31">
         <v>2.4649999999999999</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="31">
         <v>2.5190000000000001</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="31">
         <v>134.46299999999999</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="31">
         <v>134.249</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="31">
         <v>134.68299999999999</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="31">
         <v>144.11099999999999</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="31">
         <v>143.77699999999999</v>
       </c>
-      <c r="M7" s="11">
+      <c r="M7" s="31">
         <v>144.45400000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="3" customFormat="1" ht="12" customHeight="1"/>
+    <row r="8" spans="1:13" s="3" customFormat="1" ht="12" customHeight="1">
+      <c r="A8" s="32"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="33"/>
+    </row>
     <row r="9" spans="1:13" s="1" customFormat="1" ht="12" customHeight="1">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+    </row>
+    <row r="10" spans="1:13" ht="12" customHeight="1">
+      <c r="A10" s="27"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
+    </row>
+    <row r="11" spans="1:13" ht="12" customHeight="1">
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A9:M9"/>
+  <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="I9:J10"/>
+    <mergeCell ref="K9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="A9:G11"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1141,34 +1188,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="2" customFormat="1" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:9" s="2" customFormat="1" ht="12" customHeight="1">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="1:9" ht="12" customHeight="1">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:9" ht="12" customHeight="1">
       <c r="A4" s="8" t="s">
@@ -1177,10 +1224,10 @@
       <c r="B4" s="8">
         <v>1</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:9" ht="12" customHeight="1">
       <c r="A5" s="8" t="s">
@@ -1189,132 +1236,160 @@
       <c r="B5" s="8">
         <v>5</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:9" ht="12" customHeight="1">
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="12">
         <v>355.51</v>
       </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:9" ht="12" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="12">
         <v>105.4</v>
       </c>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
     </row>
     <row r="8" spans="1:9" ht="12" customHeight="1">
       <c r="A8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="12">
         <v>82.08</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
     </row>
     <row r="9" spans="1:9" ht="12" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="12">
         <v>56.05</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:9" ht="12" customHeight="1">
       <c r="A10" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="12">
         <v>53.06</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
     </row>
     <row r="11" spans="1:9" ht="12" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="12">
         <v>0.43070000000000003</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
     </row>
     <row r="12" spans="1:9" ht="12" customHeight="1">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="30">
         <v>5.7000000000000002E-3</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+    </row>
+    <row r="13" spans="1:9" ht="12" customHeight="1">
+      <c r="A13" s="35"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:9" ht="12" customHeight="1">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="31"/>
-    </row>
-    <row r="16" spans="1:9" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="17" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="18" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="19" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="20" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="21" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="22" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="23" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="24" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="25" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="26" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="27" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="28" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="29" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="30" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="31" s="4" customFormat="1" ht="12" customHeight="1"/>
-    <row r="32" s="4" customFormat="1" ht="12" customHeight="1"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+    </row>
+    <row r="15" spans="1:9" ht="12" customHeight="1">
+      <c r="A15" s="26"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" spans="1:9" s="4" customFormat="1" ht="12" customHeight="1">
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
+    </row>
+    <row r="17" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1">
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+    </row>
+    <row r="18" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1">
+      <c r="A18" s="26"/>
+      <c r="B18" s="26"/>
+    </row>
+    <row r="19" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="20" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="21" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="22" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="23" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="24" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="25" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="26" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="27" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="28" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="29" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="30" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="31" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
+    <row r="32" spans="1:2" s="4" customFormat="1" ht="12" customHeight="1"/>
     <row r="33" s="4" customFormat="1" ht="12" customHeight="1"/>
     <row r="34" s="4" customFormat="1" ht="12" customHeight="1"/>
     <row r="35" s="4" customFormat="1" ht="12" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A14:B18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1323,149 +1398,165 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06A3A1CD-BE66-9649-818B-144D364A9347}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="5" width="13.83203125" style="5" customWidth="1"/>
     <col min="6" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="12" customHeight="1">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:5" ht="12" customHeight="1">
+      <c r="A1" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="14"/>
-    </row>
-    <row r="2" spans="1:8" ht="12" customHeight="1">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="14"/>
-    </row>
-    <row r="3" spans="1:8" ht="12" customHeight="1">
-      <c r="A3" s="26" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+    </row>
+    <row r="2" spans="1:5" ht="12" customHeight="1">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+    </row>
+    <row r="3" spans="1:5" ht="12" customHeight="1">
+      <c r="A3" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="23" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="12" customHeight="1">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:5" ht="12" customHeight="1">
+      <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="13" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="12" customHeight="1">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:5" ht="12" customHeight="1">
+      <c r="A5" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="12" customHeight="1">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:5" ht="12" customHeight="1">
+      <c r="A6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="12" customHeight="1">
-      <c r="A7" s="15" t="s">
+    <row r="7" spans="1:5" ht="12" customHeight="1">
+      <c r="A7" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="12" customHeight="1">
-      <c r="A8" s="16" t="s">
+    <row r="8" spans="1:5" ht="12" customHeight="1">
+      <c r="A8" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="36" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="12" customHeight="1">
-      <c r="A10" s="31" t="s">
+    <row r="9" spans="1:5" ht="12" customHeight="1">
+      <c r="A9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+    </row>
+    <row r="10" spans="1:5" ht="12" customHeight="1">
+      <c r="A10" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-    </row>
-    <row r="12" spans="1:8" ht="12" customHeight="1">
-      <c r="B12" s="27"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+    </row>
+    <row r="11" spans="1:5" ht="12" customHeight="1">
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+    </row>
+    <row r="12" spans="1:5" ht="12" customHeight="1">
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A10:H10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A10:E12"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1481,22 +1572,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="12" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:6" ht="12" customHeight="1">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="1:6" ht="12" customHeight="1">
       <c r="A3" s="8" t="s">
@@ -1517,22 +1608,22 @@
       <c r="F4" s="8"/>
     </row>
     <row r="5" spans="1:6" ht="12" customHeight="1">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="21" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1540,19 +1631,19 @@
       <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="17">
+      <c r="B6" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="14">
         <v>62.483870967742092</v>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="14">
         <v>351.41666666666953</v>
       </c>
     </row>
@@ -1560,19 +1651,19 @@
       <c r="A7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="17" t="s">
+      <c r="B7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1580,19 +1671,19 @@
       <c r="A8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="17" t="s">
+      <c r="B8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1600,19 +1691,19 @@
       <c r="A9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="14">
         <v>96.764705882352914</v>
       </c>
-      <c r="C9" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="17">
+      <c r="C9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="14">
         <v>345.33333333333559</v>
       </c>
     </row>
@@ -1620,19 +1711,19 @@
       <c r="A10" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="15">
         <v>162.82352941176461</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="18">
+      <c r="C10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="15">
         <v>105.8709677419355</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="15" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1663,22 +1754,22 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="12" customHeight="1">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="24" t="s">
+      <c r="F14" s="21" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1686,19 +1777,19 @@
       <c r="A15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="17">
+      <c r="B15" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="14">
         <v>116.6666666666668</v>
       </c>
-      <c r="F15" s="17">
+      <c r="F15" s="14">
         <v>471.83333333334087</v>
       </c>
     </row>
@@ -1706,19 +1797,19 @@
       <c r="A16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="17" t="s">
+      <c r="B16" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1726,19 +1817,19 @@
       <c r="A17" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="17" t="s">
+      <c r="B17" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1746,19 +1837,19 @@
       <c r="A18" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="17">
+      <c r="B18" s="14">
         <v>808.50000000001069</v>
       </c>
-      <c r="C18" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="17">
+      <c r="C18" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="14">
         <v>355.16666666667368</v>
       </c>
     </row>
@@ -1766,19 +1857,19 @@
       <c r="A19" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="15">
         <v>1378.5000000000059</v>
       </c>
-      <c r="C19" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="18">
+      <c r="C19" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="15">
         <v>569.99999999999818</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="15" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1809,22 +1900,22 @@
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" ht="12" customHeight="1">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="F23" s="24" t="s">
+      <c r="F23" s="21" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1835,16 +1926,16 @@
       <c r="B24" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="14">
         <v>1294.395722</v>
       </c>
-      <c r="D24" s="17">
+      <c r="D24" s="14">
         <v>1419.395722</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F24" s="17">
+      <c r="F24" s="14">
         <v>23.395721999999999</v>
       </c>
     </row>
@@ -1852,19 +1943,19 @@
       <c r="A25" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="20">
+      <c r="C25" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="17">
         <v>125</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="20" t="s">
+      <c r="F25" s="17" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1872,19 +1963,19 @@
       <c r="A26" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="17">
         <v>1</v>
       </c>
-      <c r="D26" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="20" t="s">
+      <c r="D26" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F26" s="20" t="s">
+      <c r="F26" s="17" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1892,19 +1983,19 @@
       <c r="A27" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="17">
         <v>1301.2994650000001</v>
       </c>
-      <c r="D27" s="20">
+      <c r="D27" s="17">
         <v>1426.2994650000001</v>
       </c>
-      <c r="E27" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="20">
+      <c r="E27" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="17">
         <v>30.299465000000001</v>
       </c>
     </row>
@@ -1912,19 +2003,19 @@
       <c r="A28" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="21">
+      <c r="C28" s="18">
         <v>1271</v>
       </c>
-      <c r="D28" s="21">
+      <c r="D28" s="18">
         <v>1396</v>
       </c>
-      <c r="E28" s="21" t="s">
+      <c r="E28" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="F28" s="18" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1955,22 +2046,22 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6" ht="12" customHeight="1">
-      <c r="A32" s="24" t="s">
+      <c r="A32" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B32" s="24" t="s">
+      <c r="B32" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D32" s="24" t="s">
+      <c r="D32" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="E32" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="F32" s="24" t="s">
+      <c r="F32" s="21" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1978,19 +2069,19 @@
       <c r="A33" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B33" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C33" s="17">
+      <c r="B33" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" s="14">
         <v>473.83999999999691</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="14">
         <v>271.87313432835799</v>
       </c>
-      <c r="E33" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="17">
+      <c r="E33" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="14">
         <v>112.0799999999998</v>
       </c>
     </row>
@@ -1998,19 +2089,19 @@
       <c r="A34" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B34" s="17">
+      <c r="B34" s="14">
         <v>126.9108910891094</v>
       </c>
-      <c r="C34" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="17">
+      <c r="C34" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="14">
         <v>335.73880597015022</v>
       </c>
-      <c r="E34" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="17">
+      <c r="E34" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="14">
         <v>112.27000000000029</v>
       </c>
     </row>
@@ -2018,19 +2109,19 @@
       <c r="A35" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="17">
+      <c r="B35" s="14">
         <v>137.9207920792079</v>
       </c>
-      <c r="C35" s="17">
+      <c r="C35" s="14">
         <v>499.11999999999699</v>
       </c>
-      <c r="D35" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="17">
+      <c r="D35" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="14">
         <v>137.35999999999979</v>
       </c>
     </row>
@@ -2038,19 +2129,19 @@
       <c r="A36" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C36" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="17" t="s">
+      <c r="B36" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="14" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2058,61 +2149,61 @@
       <c r="A37" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B37" s="18">
+      <c r="B37" s="15">
         <v>56.881188118811998</v>
       </c>
-      <c r="C37" s="18">
+      <c r="C37" s="15">
         <v>361.75999999999772</v>
       </c>
-      <c r="D37" s="18">
+      <c r="D37" s="15">
         <v>244.69402985074629</v>
       </c>
-      <c r="E37" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="18" t="s">
+      <c r="E37" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="6" customFormat="1" ht="12" customHeight="1">
-      <c r="A39" s="30" t="s">
+      <c r="A39" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="30"/>
-      <c r="F39" s="30"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
     </row>
     <row r="40" spans="1:6" ht="12" customHeight="1">
-      <c r="A40" s="30"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="30"/>
+      <c r="A40" s="28"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
     </row>
     <row r="41" spans="1:6" ht="12" customHeight="1">
-      <c r="A41" s="30"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
-      <c r="E41" s="30"/>
-      <c r="F41" s="30"/>
+      <c r="A41" s="28"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
     </row>
     <row r="42" spans="1:6" ht="12" customHeight="1">
-      <c r="A42" s="30"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="30"/>
-      <c r="F42" s="30"/>
+      <c r="A42" s="28"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
     </row>
     <row r="46" spans="1:6" ht="12" customHeight="1">
-      <c r="B46" s="22"/>
+      <c r="B46" s="19"/>
     </row>
     <row r="47" spans="1:6" ht="12" customHeight="1">
-      <c r="E47" s="19"/>
+      <c r="E47" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>